<commit_message>
Add spend-vs-earn breakdown: per-SKU + 12-month ramp projection
New XLSX sheet 'Расходы_Доходы' (live formulas: order qty -> spend, UAE
sales -> revenue/EBITDA per month & year, plus 12-month ramp with launch
PPC 35% burn). New DOCX section 7.1 with the same per-SKU table and cash
summary.

Spend: ~559k AED start (417k inventory + 142k launch). Earn at full ramp:
~306k AED revenue/mo, ~73k AED EBITDA/mo (~879k/yr). Year-1 cash result
after launch burn ~+378k AED.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GAAKUQwoVwhjmCDaGhFmCq
</commit_message>
<xml_diff>
--- a/deliverables/UAE_HomeKitchen_TEO_Model_2026-07.xlsx
+++ b/deliverables/UAE_HomeKitchen_TEO_Model_2026-07.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Модель_ТЭО" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инвестиции" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Справка_FBA" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Расходы_Доходы" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="USD_AED">'Параметры'!$B$3</definedName>
@@ -145,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -219,6 +220,18 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4565,4 +4578,1274 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>СКОЛЬКО ПОТРАТИМ И СКОЛЬКО ЗАРАБОТАЕМ. Столбец 'Заказ, шт' — ввод; остальное — формулы.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>Товар</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>Заказ, шт</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>Landed AED/шт</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>ЗАКУПКА AED</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>Продажи ОАЭ/мес</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>Цена AED</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>Выручка/мес AED</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>EBITDA/шт (режим)</t>
+        </is>
+      </c>
+      <c r="J3" s="11" t="inlineStr">
+        <is>
+          <t>EBITDA/мес AED</t>
+        </is>
+      </c>
+      <c r="K3" s="11" t="inlineStr">
+        <is>
+          <t>EBITDA/мес (запуск)</t>
+        </is>
+      </c>
+      <c r="L3" s="11" t="inlineStr">
+        <is>
+          <t>EBITDA/год AED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Мини-вентилятор ручной турбо, аккумуляторный</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="n">
+        <v>600</v>
+      </c>
+      <c r="D4" s="21">
+        <f>Модель_ТЭО!N4</f>
+        <v/>
+      </c>
+      <c r="E4" s="26">
+        <f>C4*D4</f>
+        <v/>
+      </c>
+      <c r="F4" s="26">
+        <f>Модель_ТЭО!K4*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G4" s="26">
+        <f>Модель_ТЭО!F4</f>
+        <v/>
+      </c>
+      <c r="H4" s="26">
+        <f>F4*G4</f>
+        <v/>
+      </c>
+      <c r="I4" s="21">
+        <f>Модель_ТЭО!V4</f>
+        <v/>
+      </c>
+      <c r="J4" s="26">
+        <f>F4*I4</f>
+        <v/>
+      </c>
+      <c r="K4" s="26">
+        <f>F4*Модель_ТЭО!Y4</f>
+        <v/>
+      </c>
+      <c r="L4" s="26">
+        <f>J4*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Вентилятор на шею безлопастной (носимый)</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="n">
+        <v>500</v>
+      </c>
+      <c r="D5" s="21">
+        <f>Модель_ТЭО!N5</f>
+        <v/>
+      </c>
+      <c r="E5" s="26">
+        <f>C5*D5</f>
+        <v/>
+      </c>
+      <c r="F5" s="26">
+        <f>Модель_ТЭО!K5*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G5" s="26">
+        <f>Модель_ТЭО!F5</f>
+        <v/>
+      </c>
+      <c r="H5" s="26">
+        <f>F5*G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="21">
+        <f>Модель_ТЭО!V5</f>
+        <v/>
+      </c>
+      <c r="J5" s="26">
+        <f>F5*I5</f>
+        <v/>
+      </c>
+      <c r="K5" s="26">
+        <f>F5*Модель_ТЭО!Y5</f>
+        <v/>
+      </c>
+      <c r="L5" s="26">
+        <f>J5*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Портативный кондиционер/охладитель воздуха</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>300</v>
+      </c>
+      <c r="D6" s="21">
+        <f>Модель_ТЭО!N6</f>
+        <v/>
+      </c>
+      <c r="E6" s="26">
+        <f>C6*D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="26">
+        <f>Модель_ТЭО!K6*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G6" s="26">
+        <f>Модель_ТЭО!F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="26">
+        <f>F6*G6</f>
+        <v/>
+      </c>
+      <c r="I6" s="21">
+        <f>Модель_ТЭО!V6</f>
+        <v/>
+      </c>
+      <c r="J6" s="26">
+        <f>F6*I6</f>
+        <v/>
+      </c>
+      <c r="K6" s="26">
+        <f>F6*Модель_ТЭО!Y6</f>
+        <v/>
+      </c>
+      <c r="L6" s="26">
+        <f>J6*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Очиститель воздуха для дома (HEPA), большая комната</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>300</v>
+      </c>
+      <c r="D7" s="21">
+        <f>Модель_ТЭО!N7</f>
+        <v/>
+      </c>
+      <c r="E7" s="26">
+        <f>C7*D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="26">
+        <f>Модель_ТЭО!K7*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G7" s="26">
+        <f>Модель_ТЭО!F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="26">
+        <f>F7*G7</f>
+        <v/>
+      </c>
+      <c r="I7" s="21">
+        <f>Модель_ТЭО!V7</f>
+        <v/>
+      </c>
+      <c r="J7" s="26">
+        <f>F7*I7</f>
+        <v/>
+      </c>
+      <c r="K7" s="26">
+        <f>F7*Модель_ТЭО!Y7</f>
+        <v/>
+      </c>
+      <c r="L7" s="26">
+        <f>J7*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Осушитель воздуха для дома (~93 м²)</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>250</v>
+      </c>
+      <c r="D8" s="21">
+        <f>Модель_ТЭО!N8</f>
+        <v/>
+      </c>
+      <c r="E8" s="26">
+        <f>C8*D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="26">
+        <f>Модель_ТЭО!K8*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G8" s="26">
+        <f>Модель_ТЭО!F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="26">
+        <f>F8*G8</f>
+        <v/>
+      </c>
+      <c r="I8" s="21">
+        <f>Модель_ТЭО!V8</f>
+        <v/>
+      </c>
+      <c r="J8" s="26">
+        <f>F8*I8</f>
+        <v/>
+      </c>
+      <c r="K8" s="26">
+        <f>F8*Модель_ТЭО!Y8</f>
+        <v/>
+      </c>
+      <c r="L8" s="26">
+        <f>J8*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Ручной пароочиститель под давлением (110°C)</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>300</v>
+      </c>
+      <c r="D9" s="21">
+        <f>Модель_ТЭО!N9</f>
+        <v/>
+      </c>
+      <c r="E9" s="26">
+        <f>C9*D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="26">
+        <f>Модель_ТЭО!K9*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G9" s="26">
+        <f>Модель_ТЭО!F9</f>
+        <v/>
+      </c>
+      <c r="H9" s="26">
+        <f>F9*G9</f>
+        <v/>
+      </c>
+      <c r="I9" s="21">
+        <f>Модель_ТЭО!V9</f>
+        <v/>
+      </c>
+      <c r="J9" s="26">
+        <f>F9*I9</f>
+        <v/>
+      </c>
+      <c r="K9" s="26">
+        <f>F9*Модель_ТЭО!Y9</f>
+        <v/>
+      </c>
+      <c r="L9" s="26">
+        <f>J9*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Отпариватель для одежды 1000W портативный</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>300</v>
+      </c>
+      <c r="D10" s="21">
+        <f>Модель_ТЭО!N10</f>
+        <v/>
+      </c>
+      <c r="E10" s="26">
+        <f>C10*D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="26">
+        <f>Модель_ТЭО!K10*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G10" s="26">
+        <f>Модель_ТЭО!F10</f>
+        <v/>
+      </c>
+      <c r="H10" s="26">
+        <f>F10*G10</f>
+        <v/>
+      </c>
+      <c r="I10" s="21">
+        <f>Модель_ТЭО!V10</f>
+        <v/>
+      </c>
+      <c r="J10" s="26">
+        <f>F10*I10</f>
+        <v/>
+      </c>
+      <c r="K10" s="26">
+        <f>F10*Модель_ТЭО!Y10</f>
+        <v/>
+      </c>
+      <c r="L10" s="26">
+        <f>J10*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Ремни для переноски мебели (плечевые), 2 чел.</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D11" s="21">
+        <f>Модель_ТЭО!N11</f>
+        <v/>
+      </c>
+      <c r="E11" s="26">
+        <f>C11*D11</f>
+        <v/>
+      </c>
+      <c r="F11" s="26">
+        <f>Модель_ТЭО!K11*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G11" s="26">
+        <f>Модель_ТЭО!F11</f>
+        <v/>
+      </c>
+      <c r="H11" s="26">
+        <f>F11*G11</f>
+        <v/>
+      </c>
+      <c r="I11" s="21">
+        <f>Модель_ТЭО!V11</f>
+        <v/>
+      </c>
+      <c r="J11" s="26">
+        <f>F11*I11</f>
+        <v/>
+      </c>
+      <c r="K11" s="26">
+        <f>F11*Модель_ТЭО!Y11</f>
+        <v/>
+      </c>
+      <c r="L11" s="26">
+        <f>J11*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Вакуумные пакеты для хранения, 15 шт</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>500</v>
+      </c>
+      <c r="D12" s="21">
+        <f>Модель_ТЭО!N12</f>
+        <v/>
+      </c>
+      <c r="E12" s="26">
+        <f>C12*D12</f>
+        <v/>
+      </c>
+      <c r="F12" s="26">
+        <f>Модель_ТЭО!K12*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G12" s="26">
+        <f>Модель_ТЭО!F12</f>
+        <v/>
+      </c>
+      <c r="H12" s="26">
+        <f>F12*G12</f>
+        <v/>
+      </c>
+      <c r="I12" s="21">
+        <f>Модель_ТЭО!V12</f>
+        <v/>
+      </c>
+      <c r="J12" s="26">
+        <f>F12*I12</f>
+        <v/>
+      </c>
+      <c r="K12" s="26">
+        <f>F12*Модель_ТЭО!Y12</f>
+        <v/>
+      </c>
+      <c r="L12" s="26">
+        <f>J12*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Стойка для ванной телескопическая 4-ярусная (нерж.)</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>400</v>
+      </c>
+      <c r="D13" s="21">
+        <f>Модель_ТЭО!N13</f>
+        <v/>
+      </c>
+      <c r="E13" s="26">
+        <f>C13*D13</f>
+        <v/>
+      </c>
+      <c r="F13" s="26">
+        <f>Модель_ТЭО!K13*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G13" s="26">
+        <f>Модель_ТЭО!F13</f>
+        <v/>
+      </c>
+      <c r="H13" s="26">
+        <f>F13*G13</f>
+        <v/>
+      </c>
+      <c r="I13" s="21">
+        <f>Модель_ТЭО!V13</f>
+        <v/>
+      </c>
+      <c r="J13" s="26">
+        <f>F13*I13</f>
+        <v/>
+      </c>
+      <c r="K13" s="26">
+        <f>F13*Модель_ТЭО!Y13</f>
+        <v/>
+      </c>
+      <c r="L13" s="26">
+        <f>J13*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Корзина для белья с крышкой, складная 100 л</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="n">
+        <v>400</v>
+      </c>
+      <c r="D14" s="21">
+        <f>Модель_ТЭО!N14</f>
+        <v/>
+      </c>
+      <c r="E14" s="26">
+        <f>C14*D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="26">
+        <f>Модель_ТЭО!K14*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G14" s="26">
+        <f>Модель_ТЭО!F14</f>
+        <v/>
+      </c>
+      <c r="H14" s="26">
+        <f>F14*G14</f>
+        <v/>
+      </c>
+      <c r="I14" s="21">
+        <f>Модель_ТЭО!V14</f>
+        <v/>
+      </c>
+      <c r="J14" s="26">
+        <f>F14*I14</f>
+        <v/>
+      </c>
+      <c r="K14" s="26">
+        <f>F14*Модель_ТЭО!Y14</f>
+        <v/>
+      </c>
+      <c r="L14" s="26">
+        <f>J14*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Набор кухонных ножей 8 предметов (нерж., подставка)</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="n">
+        <v>400</v>
+      </c>
+      <c r="D15" s="21">
+        <f>Модель_ТЭО!N15</f>
+        <v/>
+      </c>
+      <c r="E15" s="26">
+        <f>C15*D15</f>
+        <v/>
+      </c>
+      <c r="F15" s="26">
+        <f>Модель_ТЭО!K15*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G15" s="26">
+        <f>Модель_ТЭО!F15</f>
+        <v/>
+      </c>
+      <c r="H15" s="26">
+        <f>F15*G15</f>
+        <v/>
+      </c>
+      <c r="I15" s="21">
+        <f>Модель_ТЭО!V15</f>
+        <v/>
+      </c>
+      <c r="J15" s="26">
+        <f>F15*I15</f>
+        <v/>
+      </c>
+      <c r="K15" s="26">
+        <f>F15*Модель_ТЭО!Y15</f>
+        <v/>
+      </c>
+      <c r="L15" s="26">
+        <f>J15*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Вакуумные пакеты с беспроводным электронасосом (travel)</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="n">
+        <v>300</v>
+      </c>
+      <c r="D16" s="21">
+        <f>Модель_ТЭО!N16</f>
+        <v/>
+      </c>
+      <c r="E16" s="26">
+        <f>C16*D16</f>
+        <v/>
+      </c>
+      <c r="F16" s="26">
+        <f>Модель_ТЭО!K16*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G16" s="26">
+        <f>Модель_ТЭО!F16</f>
+        <v/>
+      </c>
+      <c r="H16" s="26">
+        <f>F16*G16</f>
+        <v/>
+      </c>
+      <c r="I16" s="21">
+        <f>Модель_ТЭО!V16</f>
+        <v/>
+      </c>
+      <c r="J16" s="26">
+        <f>F16*I16</f>
+        <v/>
+      </c>
+      <c r="K16" s="26">
+        <f>F16*Модель_ТЭО!Y16</f>
+        <v/>
+      </c>
+      <c r="L16" s="26">
+        <f>J16*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Искусственная зелень эвкалипт, 130 шт (декор)</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="n">
+        <v>500</v>
+      </c>
+      <c r="D17" s="21">
+        <f>Модель_ТЭО!N17</f>
+        <v/>
+      </c>
+      <c r="E17" s="26">
+        <f>C17*D17</f>
+        <v/>
+      </c>
+      <c r="F17" s="26">
+        <f>Модель_ТЭО!K17*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G17" s="26">
+        <f>Модель_ТЭО!F17</f>
+        <v/>
+      </c>
+      <c r="H17" s="26">
+        <f>F17*G17</f>
+        <v/>
+      </c>
+      <c r="I17" s="21">
+        <f>Модель_ТЭО!V17</f>
+        <v/>
+      </c>
+      <c r="J17" s="26">
+        <f>F17*I17</f>
+        <v/>
+      </c>
+      <c r="K17" s="26">
+        <f>F17*Модель_ТЭО!Y17</f>
+        <v/>
+      </c>
+      <c r="L17" s="26">
+        <f>J17*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Офисное кресло руководителя, эко-кожа</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="n">
+        <v>120</v>
+      </c>
+      <c r="D18" s="21">
+        <f>Модель_ТЭО!N18</f>
+        <v/>
+      </c>
+      <c r="E18" s="26">
+        <f>C18*D18</f>
+        <v/>
+      </c>
+      <c r="F18" s="26">
+        <f>Модель_ТЭО!K18*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G18" s="26">
+        <f>Модель_ТЭО!F18</f>
+        <v/>
+      </c>
+      <c r="H18" s="26">
+        <f>F18*G18</f>
+        <v/>
+      </c>
+      <c r="I18" s="21">
+        <f>Модель_ТЭО!V18</f>
+        <v/>
+      </c>
+      <c r="J18" s="26">
+        <f>F18*I18</f>
+        <v/>
+      </c>
+      <c r="K18" s="26">
+        <f>F18*Модель_ТЭО!Y18</f>
+        <v/>
+      </c>
+      <c r="L18" s="26">
+        <f>J18*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Эргономичное офисное кресло (сетка), для долгой работы</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="n">
+        <v>120</v>
+      </c>
+      <c r="D19" s="21">
+        <f>Модель_ТЭО!N19</f>
+        <v/>
+      </c>
+      <c r="E19" s="26">
+        <f>C19*D19</f>
+        <v/>
+      </c>
+      <c r="F19" s="26">
+        <f>Модель_ТЭО!K19*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G19" s="26">
+        <f>Модель_ТЭО!F19</f>
+        <v/>
+      </c>
+      <c r="H19" s="26">
+        <f>F19*G19</f>
+        <v/>
+      </c>
+      <c r="I19" s="21">
+        <f>Модель_ТЭО!V19</f>
+        <v/>
+      </c>
+      <c r="J19" s="26">
+        <f>F19*I19</f>
+        <v/>
+      </c>
+      <c r="K19" s="26">
+        <f>F19*Модель_ТЭО!Y19</f>
+        <v/>
+      </c>
+      <c r="L19" s="26">
+        <f>J19*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Офисное кресло эргономичное (сетка) с подголовником</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="n">
+        <v>150</v>
+      </c>
+      <c r="D20" s="21">
+        <f>Модель_ТЭО!N20</f>
+        <v/>
+      </c>
+      <c r="E20" s="26">
+        <f>C20*D20</f>
+        <v/>
+      </c>
+      <c r="F20" s="26">
+        <f>Модель_ТЭО!K20*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G20" s="26">
+        <f>Модель_ТЭО!F20</f>
+        <v/>
+      </c>
+      <c r="H20" s="26">
+        <f>F20*G20</f>
+        <v/>
+      </c>
+      <c r="I20" s="21">
+        <f>Модель_ТЭО!V20</f>
+        <v/>
+      </c>
+      <c r="J20" s="26">
+        <f>F20*I20</f>
+        <v/>
+      </c>
+      <c r="K20" s="26">
+        <f>F20*Модель_ТЭО!Y20</f>
+        <v/>
+      </c>
+      <c r="L20" s="26">
+        <f>J20*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Кресло усиленное Big&amp;Tall (до ~180 кг), откидные подлокотники</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="n">
+        <v>80</v>
+      </c>
+      <c r="D21" s="21">
+        <f>Модель_ТЭО!N21</f>
+        <v/>
+      </c>
+      <c r="E21" s="26">
+        <f>C21*D21</f>
+        <v/>
+      </c>
+      <c r="F21" s="26">
+        <f>Модель_ТЭО!K21*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G21" s="26">
+        <f>Модель_ТЭО!F21</f>
+        <v/>
+      </c>
+      <c r="H21" s="26">
+        <f>F21*G21</f>
+        <v/>
+      </c>
+      <c r="I21" s="21">
+        <f>Модель_ТЭО!V21</f>
+        <v/>
+      </c>
+      <c r="J21" s="26">
+        <f>F21*I21</f>
+        <v/>
+      </c>
+      <c r="K21" s="26">
+        <f>F21*Модель_ТЭО!Y21</f>
+        <v/>
+      </c>
+      <c r="L21" s="26">
+        <f>J21*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Ковер 8x10 (240x300) бохо, для гостиной</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="n">
+        <v>200</v>
+      </c>
+      <c r="D22" s="21">
+        <f>Модель_ТЭО!N22</f>
+        <v/>
+      </c>
+      <c r="E22" s="26">
+        <f>C22*D22</f>
+        <v/>
+      </c>
+      <c r="F22" s="26">
+        <f>Модель_ТЭО!K22*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G22" s="26">
+        <f>Модель_ТЭО!F22</f>
+        <v/>
+      </c>
+      <c r="H22" s="26">
+        <f>F22*G22</f>
+        <v/>
+      </c>
+      <c r="I22" s="21">
+        <f>Модель_ТЭО!V22</f>
+        <v/>
+      </c>
+      <c r="J22" s="26">
+        <f>F22*I22</f>
+        <v/>
+      </c>
+      <c r="K22" s="26">
+        <f>F22*Модель_ТЭО!Y22</f>
+        <v/>
+      </c>
+      <c r="L22" s="26">
+        <f>J22*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Коврик под офисное кресло (защита пола), XL</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="n">
+        <v>200</v>
+      </c>
+      <c r="D23" s="21">
+        <f>Модель_ТЭО!N23</f>
+        <v/>
+      </c>
+      <c r="E23" s="26">
+        <f>C23*D23</f>
+        <v/>
+      </c>
+      <c r="F23" s="26">
+        <f>Модель_ТЭО!K23*UAE_MKT*SHARE</f>
+        <v/>
+      </c>
+      <c r="G23" s="26">
+        <f>Модель_ТЭО!F23</f>
+        <v/>
+      </c>
+      <c r="H23" s="26">
+        <f>F23*G23</f>
+        <v/>
+      </c>
+      <c r="I23" s="21">
+        <f>Модель_ТЭО!V23</f>
+        <v/>
+      </c>
+      <c r="J23" s="26">
+        <f>F23*I23</f>
+        <v/>
+      </c>
+      <c r="K23" s="26">
+        <f>F23*Модель_ТЭО!Y23</f>
+        <v/>
+      </c>
+      <c r="L23" s="26">
+        <f>J23*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="27" t="n"/>
+      <c r="B24" s="28" t="inlineStr">
+        <is>
+          <t>ИТОГО (20 SKU)</t>
+        </is>
+      </c>
+      <c r="C24" s="27" t="n"/>
+      <c r="D24" s="27" t="n"/>
+      <c r="E24" s="29">
+        <f>SUM(E4:E23)</f>
+        <v/>
+      </c>
+      <c r="F24" s="27" t="n"/>
+      <c r="G24" s="27" t="n"/>
+      <c r="H24" s="29">
+        <f>SUM(H4:H23)</f>
+        <v/>
+      </c>
+      <c r="I24" s="27" t="n"/>
+      <c r="J24" s="29">
+        <f>SUM(J4:J23)</f>
+        <v/>
+      </c>
+      <c r="K24" s="29">
+        <f>SUM(K4:K23)</f>
+        <v/>
+      </c>
+      <c r="L24" s="29">
+        <f>SUM(L4:L23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="31" t="inlineStr">
+        <is>
+          <t>ИТОГ: РАСХОДЫ И ДОХОДЫ</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Закупка (оборотный капитал), AED</t>
+        </is>
+      </c>
+      <c r="E27" s="41">
+        <f>E24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Бюджет запуска (единоразово), AED</t>
+        </is>
+      </c>
+      <c r="E28" s="42">
+        <f>(18000+14000+22000+60000+15000)*1.1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>ИТОГО потратим на старте, AED</t>
+        </is>
+      </c>
+      <c r="E29" s="43">
+        <f>E27+E28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Выручка/мес (полный разгон), AED</t>
+        </is>
+      </c>
+      <c r="E30" s="42">
+        <f>H24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>EBITDA/мес (полный разгон), AED</t>
+        </is>
+      </c>
+      <c r="E31" s="41">
+        <f>J24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Прибыль/мес после налога 9%, AED</t>
+        </is>
+      </c>
+      <c r="E32" s="42">
+        <f>J24*(1-CIT)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>EBITDA/год (полный разгон), AED</t>
+        </is>
+      </c>
+      <c r="E33" s="41">
+        <f>M24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="31" t="inlineStr">
+        <is>
+          <t>12-МЕСЯЧНЫЙ ПРОГНОЗ (разгон, PPC 35% в старте)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Мес 1-3 (запуск, 40% объёма)</t>
+        </is>
+      </c>
+      <c r="E36" s="42">
+        <f>L24*0.4*3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Мес 4-6 (70% объёма, режим)</t>
+        </is>
+      </c>
+      <c r="E37" s="42">
+        <f>J24*0.7*3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Мес 7-12 (100% объёма, режим)</t>
+        </is>
+      </c>
+      <c r="E38" s="42">
+        <f>J24*6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>EBITDA за 1-й год (до налога), AED</t>
+        </is>
+      </c>
+      <c r="E39" s="41">
+        <f>E36+E37+E38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>Чистая прибыль 1-го года после 9%, AED</t>
+        </is>
+      </c>
+      <c r="E40" s="44">
+        <f>E39*(1-CIT)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Денежный результат 1-го года (минус бюджет запуска), AED</t>
+        </is>
+      </c>
+      <c r="E41" s="44">
+        <f>E40-E28</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>